<commit_message>
feat: add Appearance screen and integrate content structure for appearance and dress guidelines
</commit_message>
<xml_diff>
--- a/google-sheets-template/signage-content-template.xlsx
+++ b/google-sheets-template/signage-content-template.xlsx
@@ -7,11 +7,12 @@
     <sheet sheetId="1" name="הוראות" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Ticker" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Home" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Services" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Discipline" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Procedures" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Announcements" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Safety" state="visible" r:id="rId11"/>
+    <sheet sheetId="4" name="Appearance" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Services" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Discipline" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Procedures" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Announcements" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Safety" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -48,7 +49,7 @@
 </comments>
 </file>
 
-<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Author</author>
@@ -122,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="166">
   <si>
     <t>תוכן לוח התצוגה — קובץ עריכה</t>
   </si>
@@ -163,6 +164,9 @@
     <t>•  Home — מסך הבית</t>
   </si>
   <si>
+    <t>•  Appearance — מסך הופעה ולבוש</t>
+  </si>
+  <si>
     <t>•  Procedures — מסך נהלים</t>
   </si>
   <si>
@@ -236,6 +240,39 @@
   </si>
   <si>
     <t>dailyNote</t>
+  </si>
+  <si>
+    <t>כותרת</t>
+  </si>
+  <si>
+    <t>פריט</t>
+  </si>
+  <si>
+    <t>כותרת המקטע — שורות עם אותה כותרת מקובצות יחד</t>
+  </si>
+  <si>
+    <t>פריט (בולט) אחד לכל שורה</t>
+  </si>
+  <si>
+    <t>הקדמה</t>
+  </si>
+  <si>
+    <t>המשמעת בעלת חשיבות מרבית להבטחת פעילותו התקינה של צה״ל, והיא תנאי הכרחי לביצוע מלא ויעיל של המשימות המוטלות עליו.</t>
+  </si>
+  <si>
+    <t>חיילי ומפקדי צה״ל יקפידו על הופעה מסודרת ותקנית בכל עת.</t>
+  </si>
+  <si>
+    <t>הוראות הלבוש לבאים במחנות צה״ל</t>
+  </si>
+  <si>
+    <t>לא תותר כניסה בלבוש לא הולם למחנות צה״ל או באופן שאינו מכבד את כללי השירות המשותף.</t>
+  </si>
+  <si>
+    <t>חייל יקפיד על כלל הוראות הקבע של הופעה ולבוש בצורה תקנית ומסודרת.</t>
+  </si>
+  <si>
+    <t>חייל ילבש מדי שירות בכל עת שהוא בתפקיד או במסגרת צבאית, מבין פריטי הלבוש שקיבל מצה״ל ומפורטים בתעודת ציודו האישי (טופס 1004) בלבד, אלא אם נקבע אחרת בפקודות הצבא או לפיהן.</t>
   </si>
   <si>
     <t>שם</t>
@@ -338,9 +375,6 @@
     <t>המחסן המרכזי</t>
   </si>
   <si>
-    <t>כותרת</t>
-  </si>
-  <si>
     <t>תת_כותרת</t>
   </si>
   <si>
@@ -356,16 +390,16 @@
     <t>פריט לכל שורה (Alt+Enter למעבר שורה)</t>
   </si>
   <si>
-    <t>הופעה ולבוש</t>
-  </si>
-  <si>
-    <t>מדי אלף — מגולח, מהודק, מגוהץ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">תספורת תקנית לפי נהלי צה״ל
-נעליים מצוחצחות ואחידות נקיות
-תגיות שם על כל פריט ביגוד
-בדיקות הופעה מתקיימות מדי יום</t>
+    <t>היתר גידול זקן</t>
+  </si>
+  <si>
+    <t>ההיתר תקף לכל משך השירות, בכפוף לעמידה בקריטריונים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">גידול זקן מותר בהתאם לרצון הפרט, ובלבד שהוא מסודר והולם הופעה צבאית נאותה
+זקן מלא מהפאות עד הסנטר (כולל שפם), ללא ביצוע “מדרגות”
+מותר לסדר את הזקן והשפם, אך אין לקצצו עד כדי זיפים
+חובה למלא הצהרה; פגיעה בנראות הזקן תוביל לשלילת ההיתר</t>
   </si>
   <si>
     <t>דלת פתוחה</t>
@@ -1091,7 +1125,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:B23"/>
+  <dimension ref="B1:B24"/>
   <sheetFormatPr defaultRowHeight="20" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1193,24 +1227,29 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" ht="8" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+    <row r="20" ht="22" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
+    <row r="22" ht="26" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1229,42 +1268,42 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1284,39 +1323,39 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>2</v>
@@ -1330,6 +1369,77 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="90" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
@@ -1342,128 +1452,128 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="8" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1477,7 +1587,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
@@ -1489,68 +1599,68 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" ht="66" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" ht="66" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" ht="66" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1559,7 +1669,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
@@ -1570,90 +1680,90 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1663,7 +1773,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
@@ -1675,178 +1785,178 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1863,7 +1973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
@@ -1878,59 +1988,59 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" ht="96" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>2</v>
@@ -1938,42 +2048,42 @@
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" ht="96" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>2</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add installation guide, enhance Procedures and Appearance screens, and implement desktop launch scripts for Windows and macOS
</commit_message>
<xml_diff>
--- a/google-sheets-template/signage-content-template.xlsx
+++ b/google-sheets-template/signage-content-template.xlsx
@@ -100,21 +100,63 @@
     <comment ref="A9" authorId="0">
       <text>
         <r>
-          <t>סמים ואלכוהול — פסקה ראשונה</t>
+          <t>יוהל״ם — טקסט הסבר נוסף</t>
         </r>
       </text>
     </comment>
     <comment ref="A10" authorId="0">
       <text>
         <r>
-          <t>סמים ואלכוהול — פסקה שנייה</t>
+          <t>סמים ואלכוהול — פסקה ראשונה</t>
         </r>
       </text>
     </comment>
     <comment ref="A11" authorId="0">
       <text>
         <r>
-          <t>ביטחון מידע — פסקה</t>
+          <t>סמים ואלכוהול — פסקה שנייה</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A12" authorId="0">
+      <text>
+        <r>
+          <t>סמים ואלכוהול — פסקה שלישית</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="0">
+      <text>
+        <r>
+          <t>ביטחון מידע — פסקה ראשונה</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A14" authorId="0">
+      <text>
+        <r>
+          <t>ביטחון מידע — פסקה שנייה</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A15" authorId="0">
+      <text>
+        <r>
+          <t>ביטחון מידע — פסקה שלישית</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A16" authorId="0">
+      <text>
+        <r>
+          <t>ביטחון מידע — פסקה רביעית</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A17" authorId="0">
+      <text>
+        <r>
+          <t>ביטחון מידע — פסקה חמישית</t>
         </r>
       </text>
     </comment>
@@ -123,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="178">
   <si>
     <t>תוכן לוח התצוגה — קובץ עריכה</t>
   </si>
@@ -474,6 +516,12 @@
     <t>אפס סובלנות</t>
   </si>
   <si>
+    <t>card2.intro</t>
+  </si>
+  <si>
+    <t>ממונת יוהל״ם ביחידה, קצינת הת״ש - 058-7303090</t>
+  </si>
+  <si>
     <t>card2.para1</t>
   </si>
   <si>
@@ -486,10 +534,40 @@
     <t>אין למכור במתקני צה״ל משקאות אלכוהוליים לצריכה בתוך המחנות.</t>
   </si>
   <si>
+    <t>card2.para3</t>
+  </si>
+  <si>
+    <t>יש לדווח על כל נושא חריג בנושא זה למפקד הישיר ולרנ״ג הפיקוד.</t>
+  </si>
+  <si>
     <t>card3.para1</t>
   </si>
   <si>
     <t>מידע צבאי מסווג לא יועבר בטלפון / בפקס האזרחי ו/או המטכ״לי.</t>
+  </si>
+  <si>
+    <t>card3.para2</t>
+  </si>
+  <si>
+    <t>אין לחבר חיבור חיצוני למחשבים צבאיים (USB, וכו׳)</t>
+  </si>
+  <si>
+    <t>card3.para3</t>
+  </si>
+  <si>
+    <t>אין להוציא מידע צבאי מחוץ לתחומי הבסיס ללא אישור ביטחון מידע.</t>
+  </si>
+  <si>
+    <t>card3.para4</t>
+  </si>
+  <si>
+    <t>בסיום השירות במסמכים צבאיים, יש לגרוס ואין לזרוק לאשפה.</t>
+  </si>
+  <si>
+    <t>card3.para5</t>
+  </si>
+  <si>
+    <t>אין להעלות פרטים מסווגים/צבאיים על גבי רשתות חברתיות.</t>
   </si>
   <si>
     <t>מקטע</t>
@@ -1671,7 +1749,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1764,6 +1842,54 @@
       </c>
       <c r="B11" s="7" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1785,178 +1911,178 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>39</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1994,53 +2120,53 @@
         <v>80</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>81</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>83</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" ht="96" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>2</v>
@@ -2048,42 +2174,42 @@
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" ht="96" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>2</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>